<commit_message>
verification: problem 10's refinement returns the same bracket, and the row locks at 1.037
The one row of the corpus whose bracket decided on every trial and whose
refinement had never been run. At a 2D size of 2.1 m the finer mesh returns the
corpus bracket edge for edge, all nine trials decide on both meshes, and the row
locks at 1.037 against UDEC's 1.03.

The two brackets reach that answer differently: on the corpus mesh every trial
converges or diverges on its own, while on the finer one all five standing
trials are settled by the Newton corrector at 300 sweeps.

Also drops the three EXTRA_CASES entries r17's locks superseded (RJ-4, RJ-7,
RJ-15), which the figure audit had been reporting.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj010.xlsx
+++ b/docs/verification/files/rocscience/joints/rj010.xlsx
@@ -3374,7 +3374,9 @@
       <c r="G16" t="s">
         <v>34</v>
       </c>
-      <c r="D16"/>
+      <c r="D16">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>

</xml_diff>